<commit_message>
Corregimos el excel de la dimensión social
</commit_message>
<xml_diff>
--- a/data/processed/indicadores_SOC_SIEPAC.xlsx
+++ b/data/processed/indicadores_SOC_SIEPAC.xlsx
@@ -985,19 +985,19 @@
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>0.001674700183943291</v>
+        <v>1.674700183943275</v>
       </c>
       <c r="C6" s="7" t="n">
-        <v>0.001704469904945673</v>
+        <v>1.704469904945673</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>0.001676745166674422</v>
+        <v>1.676745166674422</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>0.00169191796099463</v>
+        <v>1.69191796099463</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>0.001701856994641966</v>
+        <v>1.701856994641966</v>
       </c>
     </row>
     <row r="7">
@@ -1029,19 +1029,19 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>3.629698996419138</v>
+        <v>8.711277591405931</v>
       </c>
       <c r="C8" s="7" t="n">
-        <v>3.029175503007524</v>
+        <v>7.270021207218058</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>2.95066870659458</v>
+        <v>7.08160489582699</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>2.535527284910263</v>
+        <v>6.085265483784632</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>2.214336134299205</v>
+        <v>5.314406722318093</v>
       </c>
     </row>
     <row r="9">
@@ -1073,19 +1073,19 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>3.290942100000229</v>
+        <v>4.416709446457916</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>3.065208624391028</v>
+        <v>4.055810480932906</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>3.106351586979381</v>
+        <v>4.074019022102741</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>3.032350310461753</v>
+        <v>3.905677684113087</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>3.091759270974054</v>
+        <v>3.891796891918423</v>
       </c>
     </row>
   </sheetData>
@@ -1197,19 +1197,19 @@
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>0.006225959217700948</v>
+        <v>6.22595921770089</v>
       </c>
       <c r="C6" s="7" t="n">
-        <v>0.006336632800148852</v>
+        <v>6.336632800148852</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>0.006233561760058678</v>
+        <v>6.233561760058678</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>0.006289968990177774</v>
+        <v>6.289968990177773</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>0.006326918898432973</v>
+        <v>6.326918898432972</v>
       </c>
     </row>
     <row r="7">
@@ -1241,19 +1241,19 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>9.497326752261355</v>
+        <v>22.79360082023156</v>
       </c>
       <c r="C8" s="7" t="n">
-        <v>7.926020744527325</v>
+        <v>19.02246365279723</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>7.720602967862492</v>
+        <v>18.52946062943986</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>6.634360352696893</v>
+        <v>15.9224764527489</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>5.793944298831981</v>
+        <v>13.90547645323327</v>
       </c>
     </row>
     <row r="9">
@@ -1285,19 +1285,19 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>22.23950903338138</v>
+        <v>25.49217692112361</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>21.16114533575594</v>
+        <v>24.06560184835905</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>22.61410963655608</v>
+        <v>25.45347394653541</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>22.57852348242082</v>
+        <v>25.17382266929409</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>24.68762740427068</v>
+        <v>27.09298142659333</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Corregimos datos en la dimension social, SOC2 ES
</commit_message>
<xml_diff>
--- a/data/processed/indicadores_SOC_SIEPAC.xlsx
+++ b/data/processed/indicadores_SOC_SIEPAC.xlsx
@@ -963,19 +963,19 @@
         </is>
       </c>
       <c r="B5" s="7" t="n">
-        <v>6.18992678570214</v>
+        <v>2.063308928567357</v>
       </c>
       <c r="C5" s="7" t="n">
-        <v>6.093497221687183</v>
+        <v>2.031165740562394</v>
       </c>
       <c r="D5" s="7" t="n">
-        <v>5.595099691236247</v>
+        <v>1.865033230412082</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>5.1863096066683</v>
+        <v>1.728769868889434</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>5.278357503398404</v>
+        <v>1.759452501132801</v>
       </c>
     </row>
     <row r="6">
@@ -1051,19 +1051,19 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>2.416622630946807</v>
+        <v>0.8055408769822704</v>
       </c>
       <c r="C9" s="7" t="n">
-        <v>2.252187570882236</v>
+        <v>0.7507291902940787</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>2.400984229520648</v>
+        <v>0.8003280765068828</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>2.346501664381798</v>
+        <v>0.7821672214605995</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>2.61879044419974</v>
+        <v>0.8729301480665801</v>
       </c>
     </row>
     <row r="10">
@@ -1073,19 +1073,19 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>4.416709446457916</v>
+        <v>3.460426177941363</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>4.055810480932906</v>
+        <v>3.128512170647415</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>4.074019022102741</v>
+        <v>3.185565253129752</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>3.905677684113087</v>
+        <v>3.068698653996409</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>3.891796891918423</v>
+        <v>3.014336008851963</v>
       </c>
     </row>
   </sheetData>
@@ -1175,19 +1175,19 @@
         </is>
       </c>
       <c r="B5" s="7" t="n">
-        <v>21.72650072973297</v>
+        <v>7.2421669099111</v>
       </c>
       <c r="C5" s="7" t="n">
-        <v>22.66387232801</v>
+        <v>7.554624109336666</v>
       </c>
       <c r="D5" s="7" t="n">
-        <v>21.026279414898</v>
+        <v>7.008759804965998</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>20.74355638031428</v>
+        <v>6.914518793438093</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>21.70361037554047</v>
+        <v>7.234536791846826</v>
       </c>
     </row>
     <row r="6">
@@ -1263,19 +1263,19 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>31.40490513181162</v>
+        <v>10.4683017106039</v>
       </c>
       <c r="C9" s="7" t="n">
-        <v>29.27843752653015</v>
+        <v>9.759479175510052</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>30.37673705619569</v>
+        <v>10.1255790187319</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>26.87122889154614</v>
+        <v>8.957076297182045</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>33.15575667431635</v>
+        <v>11.05191889143878</v>
       </c>
     </row>
     <row r="10">
@@ -1285,19 +1285,19 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>25.49217692112361</v>
+        <v>19.58868738095201</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>24.06560184835905</v>
+        <v>18.29423408674348</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>25.45347394653541</v>
+        <v>19.74202767196945</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>25.17382266929409</v>
+        <v>19.88329097242071</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>27.09298142659333</v>
+        <v>20.99749619883145</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Corregimos datos en SOCs - SOC2 PAN
</commit_message>
<xml_diff>
--- a/data/processed/indicadores_SOC_SIEPAC.xlsx
+++ b/data/processed/indicadores_SOC_SIEPAC.xlsx
@@ -729,19 +729,19 @@
         </is>
       </c>
       <c r="B4" s="7" t="n">
-        <v>0.5999999999999943</v>
+        <v>0.599999999999994</v>
       </c>
       <c r="C4" s="7" t="n">
-        <v>0.5999999999999943</v>
+        <v>0.599999999999994</v>
       </c>
       <c r="D4" s="7" t="n">
-        <v>0.5999999999999943</v>
+        <v>0.599999999999994</v>
       </c>
       <c r="E4" s="7" t="n">
-        <v>0.5999999999999943</v>
+        <v>0.599999999999994</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>0.5999999999999943</v>
+        <v>0.599999999999994</v>
       </c>
     </row>
     <row r="5">
@@ -751,19 +751,19 @@
         </is>
       </c>
       <c r="B5" s="7" t="n">
-        <v>2.200000000000003</v>
+        <v>2.2</v>
       </c>
       <c r="C5" s="7" t="n">
-        <v>2.099999999999994</v>
+        <v>2.09999999999999</v>
       </c>
       <c r="D5" s="7" t="n">
-        <v>1.799999999999997</v>
+        <v>1.8</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>1.700000000000003</v>
+        <v>1.7</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>1.700000000000003</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="6">
@@ -773,10 +773,10 @@
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>10.09999999999999</v>
+        <v>10.1</v>
       </c>
       <c r="C6" s="7" t="n">
-        <v>10.73999999999999</v>
+        <v>10.74</v>
       </c>
       <c r="D6" s="7" t="n">
         <v>10.06</v>
@@ -820,16 +820,16 @@
         <v>1.5</v>
       </c>
       <c r="C8" s="7" t="n">
-        <v>0.9099999999999966</v>
+        <v>0.909999999999997</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>0.7399999999999949</v>
+        <v>0.739999999999995</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>0.5900000000000034</v>
+        <v>0.590000000000003</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>0.4429999999999978</v>
+        <v>0.442999999999998</v>
       </c>
     </row>
     <row r="9">
@@ -839,16 +839,16 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>5.599999999999994</v>
+        <v>5.59999999999999</v>
       </c>
       <c r="C9" s="7" t="n">
-        <v>5.099999999999994</v>
+        <v>5.09999999999999</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>4.799999999999997</v>
+        <v>4.8</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>4.400000000000006</v>
+        <v>4.40000000000001</v>
       </c>
       <c r="F9" s="7" t="n">
         <v>4</v>
@@ -861,13 +861,13 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>5.796666666666664</v>
+        <v>5.796666666666663</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>5.61333333333333</v>
+        <v>5.613333333333329</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>5.394999999999999</v>
+        <v>5.394999999999997</v>
       </c>
       <c r="E10" s="9" t="n">
         <v>5.103333333333334</v>
@@ -985,19 +985,19 @@
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>1.674700183943275</v>
+        <v>2.343494150586636</v>
       </c>
       <c r="C6" s="7" t="n">
-        <v>1.704469904945673</v>
+        <v>2.385152453190655</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>1.676745166674422</v>
+        <v>2.346355800160955</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>1.69191796099463</v>
+        <v>2.367587872073516</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>1.701856994641966</v>
+        <v>2.38149607333744</v>
       </c>
     </row>
     <row r="7">
@@ -1007,19 +1007,19 @@
         </is>
       </c>
       <c r="B7" s="7" t="n">
-        <v>5.099601325768251</v>
+        <v>5.099601325768182</v>
       </c>
       <c r="C7" s="7" t="n">
         <v>5.138073760128728</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>5.884758195642447</v>
+        <v>5.88475819564244</v>
       </c>
       <c r="E7" s="7" t="n">
         <v>6.297761850587959</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>6.551976629698161</v>
+        <v>6.551976629698165</v>
       </c>
     </row>
     <row r="8">
@@ -1051,19 +1051,19 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>0.8055408769822704</v>
+        <v>2.599182845696212</v>
       </c>
       <c r="C9" s="7" t="n">
-        <v>0.7507291902940787</v>
+        <v>2.410129527017159</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>0.8003280765068828</v>
+        <v>2.581874243776133</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0.7821672214605995</v>
+        <v>2.52028729842289</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>0.8729301480665801</v>
+        <v>2.788155785203608</v>
       </c>
     </row>
     <row r="10">
@@ -1073,19 +1073,19 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>3.460426177941363</v>
+        <v>3.870832167167569</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>3.128512170647415</v>
+        <v>3.518525984808759</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>3.185565253129752</v>
+        <v>3.594091386589048</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>3.068698653996409</v>
+        <v>3.470996985336605</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>3.014336008851963</v>
+        <v>3.446813461490714</v>
       </c>
     </row>
   </sheetData>
@@ -1197,19 +1197,19 @@
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>6.22595921770089</v>
+        <v>8.647684382973296</v>
       </c>
       <c r="C6" s="7" t="n">
-        <v>6.336632800148852</v>
+        <v>8.801406914245572</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>6.233561760058678</v>
+        <v>8.658244103093434</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>6.289968990177773</v>
+        <v>8.736592178615814</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>6.326918898432972</v>
+        <v>8.787914574635099</v>
       </c>
     </row>
     <row r="7">
@@ -1219,19 +1219,19 @@
         </is>
       </c>
       <c r="B7" s="7" t="n">
-        <v>49.08269257595933</v>
+        <v>49.08269257595922</v>
       </c>
       <c r="C7" s="7" t="n">
-        <v>51.34316205900213</v>
+        <v>51.34316205900203</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>61.73254233847679</v>
+        <v>61.73254233847681</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>65.87033548278535</v>
+        <v>65.87033548278512</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>73.4946295223331</v>
+        <v>73.49462952233317</v>
       </c>
     </row>
     <row r="8">
@@ -1263,19 +1263,19 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>10.4683017106039</v>
+        <v>30.30085032490308</v>
       </c>
       <c r="C9" s="7" t="n">
-        <v>9.759479175510052</v>
+        <v>28.08948488981295</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>10.1255790187319</v>
+        <v>28.69401070614894</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>8.957076297182045</v>
+        <v>25.62292108637144</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>11.05191889143878</v>
+        <v>30.98654883519867</v>
       </c>
     </row>
     <row r="10">
@@ -1285,19 +1285,19 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>19.58868738095201</v>
+        <v>23.29773301088059</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>18.29423408674348</v>
+        <v>21.76003072481006</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>19.74202767196945</v>
+        <v>23.24088001037809</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>19.88329097242071</v>
+        <v>23.06870230202525</v>
       </c>
       <c r="F10" s="9" t="n">
-        <v>20.99749619883145</v>
+        <v>24.73010046882513</v>
       </c>
     </row>
   </sheetData>
@@ -1377,7 +1377,7 @@
         <v>94.33775084566619</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>88.8717968238078</v>
+        <v>88.87179682380781</v>
       </c>
     </row>
     <row r="5">
@@ -1396,10 +1396,10 @@
         <v>74.59995103887134</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>58.78355940525261</v>
+        <v>58.78355940525262</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>66.59286994597188</v>
+        <v>66.59286994597186</v>
       </c>
     </row>
     <row r="6">
@@ -1415,13 +1415,13 @@
         <v>60.0935427865742</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>65.07612850013156</v>
+        <v>65.07612850013152</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>55.77213851154134</v>
+        <v>55.77213851154131</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>50.25085859008419</v>
+        <v>50.2508585900842</v>
       </c>
     </row>
     <row r="7">
@@ -1434,16 +1434,16 @@
         <v>38.63471126652675</v>
       </c>
       <c r="C7" s="7" t="n">
-        <v>45.88832516582504</v>
+        <v>45.88832516582501</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>44.53876283005371</v>
+        <v>44.53876283005372</v>
       </c>
       <c r="E7" s="7" t="n">
         <v>39.67071028192908</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>40.13015546029065</v>
+        <v>40.13015546029064</v>
       </c>
     </row>
     <row r="8">
@@ -1453,13 +1453,13 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>50.91410095120624</v>
+        <v>50.91410095120618</v>
       </c>
       <c r="C8" s="7" t="n">
         <v>50.47289416229471</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>47.84487225862026</v>
+        <v>47.84487225862024</v>
       </c>
       <c r="E8" s="7" t="n">
         <v>42.70851717210358</v>
@@ -1497,16 +1497,16 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>64.0638344566235</v>
+        <v>64.06383445662348</v>
       </c>
       <c r="C10" s="9" t="n">
         <v>65.80089442385021</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>65.14050815451024</v>
+        <v>65.14050815451021</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>57.08690847805255</v>
+        <v>57.08690847805254</v>
       </c>
       <c r="F10" s="9" t="n">
         <v>59.14617154812704</v>
@@ -1589,7 +1589,7 @@
         <v>94.33775084566619</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>88.8717968238078</v>
+        <v>88.87179682380781</v>
       </c>
     </row>
     <row r="5">
@@ -1611,7 +1611,7 @@
         <v>60.48743069236139</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>67.14436369293645</v>
+        <v>67.14436369293644</v>
       </c>
     </row>
     <row r="6">
@@ -1627,13 +1627,13 @@
         <v>69.3002732134959</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>75.88299460484656</v>
+        <v>75.8829946048465</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>64.31680106259697</v>
+        <v>64.31680106259691</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>57.61546352765392</v>
+        <v>57.61546352765393</v>
       </c>
     </row>
     <row r="7">
@@ -1646,16 +1646,16 @@
         <v>54.84320614055069</v>
       </c>
       <c r="C7" s="7" t="n">
-        <v>58.37024562485339</v>
+        <v>58.37024562485334</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>56.51225593946253</v>
+        <v>56.51225593946255</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>49.34279731194104</v>
+        <v>49.34279731194102</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>49.20733907210177</v>
+        <v>49.20733907210176</v>
       </c>
     </row>
     <row r="8">
@@ -1665,13 +1665,13 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>69.80271586400637</v>
+        <v>69.80271586400629</v>
       </c>
       <c r="C8" s="7" t="n">
         <v>69.1978258325949</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>65.59483446479334</v>
+        <v>65.59483446479332</v>
       </c>
       <c r="E8" s="7" t="n">
         <v>58.55294375117026</v>
@@ -1712,13 +1712,13 @@
         <v>74.16244546297617</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>74.76991861026393</v>
+        <v>74.76991861026391</v>
       </c>
       <c r="D10" s="9" t="n">
         <v>73.5239033540568</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>63.61292652972094</v>
+        <v>63.61292652972093</v>
       </c>
       <c r="F10" s="9" t="n">
         <v>64.60692967954809</v>
@@ -1802,7 +1802,7 @@
         <v>2020</v>
       </c>
       <c r="C4" s="11" t="n">
-        <v>0.5999999999999943</v>
+        <v>0.599999999999994</v>
       </c>
       <c r="D4" s="11" t="n">
         <v>99.79425867013732</v>
@@ -1824,7 +1824,7 @@
         <v>2021</v>
       </c>
       <c r="C5" s="11" t="n">
-        <v>0.5999999999999943</v>
+        <v>0.599999999999994</v>
       </c>
       <c r="D5" s="11" t="n">
         <v>99.97719552064747</v>
@@ -1846,7 +1846,7 @@
         <v>2022</v>
       </c>
       <c r="C6" s="11" t="n">
-        <v>0.5999999999999943</v>
+        <v>0.599999999999994</v>
       </c>
       <c r="D6" s="11" t="n">
         <v>99.26847897567855</v>
@@ -1868,7 +1868,7 @@
         <v>2023</v>
       </c>
       <c r="C7" s="11" t="n">
-        <v>0.5999999999999943</v>
+        <v>0.599999999999994</v>
       </c>
       <c r="D7" s="11" t="n">
         <v>94.90719400972453</v>
@@ -1890,10 +1890,10 @@
         <v>2024</v>
       </c>
       <c r="C8" s="11" t="n">
-        <v>0.5999999999999943</v>
+        <v>0.599999999999994</v>
       </c>
       <c r="D8" s="11" t="n">
-        <v>89.4082463016175</v>
+        <v>89.40824630161751</v>
       </c>
       <c r="E8" s="11" t="n">
         <v>99.40000000000001</v>
@@ -1912,7 +1912,7 @@
         <v>2020</v>
       </c>
       <c r="C9" s="11" t="n">
-        <v>2.200000000000003</v>
+        <v>2.2</v>
       </c>
       <c r="D9" s="11" t="n">
         <v>83.98969544323815</v>
@@ -1934,10 +1934,10 @@
         <v>2021</v>
       </c>
       <c r="C10" s="11" t="n">
-        <v>2.099999999999994</v>
+        <v>2.09999999999999</v>
       </c>
       <c r="D10" s="11" t="n">
-        <v>84.20375203717359</v>
+        <v>84.2037520371736</v>
       </c>
       <c r="E10" s="11" t="n">
         <v>95.59999999999999</v>
@@ -1956,7 +1956,7 @@
         <v>2022</v>
       </c>
       <c r="C11" s="11" t="n">
-        <v>1.799999999999997</v>
+        <v>1.8</v>
       </c>
       <c r="D11" s="11" t="n">
         <v>77.38584132663001</v>
@@ -1978,10 +1978,10 @@
         <v>2023</v>
       </c>
       <c r="C12" s="11" t="n">
-        <v>1.700000000000003</v>
+        <v>1.7</v>
       </c>
       <c r="D12" s="11" t="n">
-        <v>60.8525459681704</v>
+        <v>60.85254596817041</v>
       </c>
       <c r="E12" s="11" t="n">
         <v>96.59999999999999</v>
@@ -2000,10 +2000,10 @@
         <v>2024</v>
       </c>
       <c r="C13" s="11" t="n">
-        <v>1.700000000000003</v>
+        <v>1.7</v>
       </c>
       <c r="D13" s="11" t="n">
-        <v>68.93671837057131</v>
+        <v>68.93671837057128</v>
       </c>
       <c r="E13" s="11" t="n">
         <v>96.59999999999999</v>
@@ -2022,7 +2022,7 @@
         <v>2020</v>
       </c>
       <c r="C14" s="11" t="n">
-        <v>10.09999999999999</v>
+        <v>10.1</v>
       </c>
       <c r="D14" s="11" t="n">
         <v>75.27843098172775</v>
@@ -2044,7 +2044,7 @@
         <v>2021</v>
       </c>
       <c r="C15" s="11" t="n">
-        <v>10.73999999999999</v>
+        <v>10.74</v>
       </c>
       <c r="D15" s="11" t="n">
         <v>71.37000330947055</v>
@@ -2069,7 +2069,7 @@
         <v>10.06</v>
       </c>
       <c r="D16" s="11" t="n">
-        <v>78.31062394721006</v>
+        <v>78.31062394721002</v>
       </c>
       <c r="E16" s="11" t="n">
         <v>83.09999999999999</v>
@@ -2091,7 +2091,7 @@
         <v>9.609999999999999</v>
       </c>
       <c r="D17" s="11" t="n">
-        <v>66.23769419422962</v>
+        <v>66.23769419422958</v>
       </c>
       <c r="E17" s="11" t="n">
         <v>84.2</v>
@@ -2113,7 +2113,7 @@
         <v>9.109999999999999</v>
       </c>
       <c r="D18" s="11" t="n">
-        <v>59.15345331381305</v>
+        <v>59.15345331381307</v>
       </c>
       <c r="E18" s="11" t="n">
         <v>84.95</v>
@@ -2157,7 +2157,7 @@
         <v>14.23</v>
       </c>
       <c r="D20" s="11" t="n">
-        <v>61.66956748531789</v>
+        <v>61.66956748531784</v>
       </c>
       <c r="E20" s="11" t="n">
         <v>74.41</v>
@@ -2179,7 +2179,7 @@
         <v>14.37</v>
       </c>
       <c r="D21" s="11" t="n">
-        <v>59.80765788915497</v>
+        <v>59.80765788915499</v>
       </c>
       <c r="E21" s="11" t="n">
         <v>74.47</v>
@@ -2201,7 +2201,7 @@
         <v>13.72</v>
       </c>
       <c r="D22" s="11" t="n">
-        <v>52.25330648304674</v>
+        <v>52.25330648304672</v>
       </c>
       <c r="E22" s="11" t="n">
         <v>75.92</v>
@@ -2245,7 +2245,7 @@
         <v>1.5</v>
       </c>
       <c r="D24" s="11" t="n">
-        <v>69.80271586400637</v>
+        <v>69.80271586400629</v>
       </c>
       <c r="E24" s="11" t="n">
         <v>72.94</v>
@@ -2264,7 +2264,7 @@
         <v>2021</v>
       </c>
       <c r="C25" s="11" t="n">
-        <v>0.9099999999999966</v>
+        <v>0.909999999999997</v>
       </c>
       <c r="D25" s="11" t="n">
         <v>69.1978258325949</v>
@@ -2286,10 +2286,10 @@
         <v>2022</v>
       </c>
       <c r="C26" s="11" t="n">
-        <v>0.7399999999999949</v>
+        <v>0.739999999999995</v>
       </c>
       <c r="D26" s="11" t="n">
-        <v>65.59483446479334</v>
+        <v>65.59483446479332</v>
       </c>
       <c r="E26" s="11" t="n">
         <v>72.94</v>
@@ -2308,7 +2308,7 @@
         <v>2023</v>
       </c>
       <c r="C27" s="11" t="n">
-        <v>0.5900000000000034</v>
+        <v>0.590000000000003</v>
       </c>
       <c r="D27" s="11" t="n">
         <v>58.55294375117026</v>
@@ -2330,7 +2330,7 @@
         <v>2024</v>
       </c>
       <c r="C28" s="11" t="n">
-        <v>0.4429999999999978</v>
+        <v>0.442999999999998</v>
       </c>
       <c r="D28" s="11" t="n">
         <v>51.80150021325011</v>
@@ -2352,7 +2352,7 @@
         <v>2020</v>
       </c>
       <c r="C29" s="11" t="n">
-        <v>5.599999999999994</v>
+        <v>5.59999999999999</v>
       </c>
       <c r="D29" s="11" t="n">
         <v>65.0397256367866</v>
@@ -2374,7 +2374,7 @@
         <v>2021</v>
       </c>
       <c r="C30" s="11" t="n">
-        <v>5.099999999999994</v>
+        <v>5.09999999999999</v>
       </c>
       <c r="D30" s="11" t="n">
         <v>68.52457386579727</v>
@@ -2396,7 +2396,7 @@
         <v>2022</v>
       </c>
       <c r="C31" s="11" t="n">
-        <v>4.799999999999997</v>
+        <v>4.8</v>
       </c>
       <c r="D31" s="11" t="n">
         <v>67.3441604373496</v>
@@ -2418,7 +2418,7 @@
         <v>2023</v>
       </c>
       <c r="C32" s="11" t="n">
-        <v>4.400000000000006</v>
+        <v>4.40000000000001</v>
       </c>
       <c r="D32" s="11" t="n">
         <v>54.69453004463444</v>

</xml_diff>